<commit_message>
Removed explicitly defined sanctions from Law cards
</commit_message>
<xml_diff>
--- a/ShiftingSands.xlsx
+++ b/ShiftingSands.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/736bb1ccd5622dcc/Documents/BoardGames/ShiftingSands/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4709" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{43E468BA-BB90-408B-BE7A-5A8C3FE17CC2}"/>
+  <xr:revisionPtr revIDLastSave="4739" documentId="11_0B1D56BE9CDCCE836B02CE7A5FB0D4A9BBFD1C62" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6F7C9001-ABB5-474D-8310-7CB85E30C8A9}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -670,94 +670,94 @@
     <t>Law HTML Description</t>
   </si>
   <si>
-    <t>The Royal Bank must have at least $L6 Coins or all Players suffer sanctions on Undermarket Actions</t>
-  </si>
-  <si>
-    <t>The Royal Bank may not have more than $L6 Coins or all Players suffer sanctions on Undermarket Actions</t>
-  </si>
-  <si>
-    <t>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions on Commission</t>
-  </si>
-  <si>
-    <t>No Player may have more than 3 + $L6 Investments or they will suffer sanctions on Commission</t>
-  </si>
-  <si>
-    <t>Each Player must deploy at least $L6 Troops or they will suffer sanctions on Petition</t>
-  </si>
-  <si>
-    <t>No Player may deploy more than $L6 Troops or they will suffer sanctions on Petition</t>
-  </si>
-  <si>
-    <t>Each Player must have at least $L6 sponsored Laws in the Edicts or in the Queue or they will suffer sanctions on Tax</t>
-  </si>
-  <si>
-    <t>No Player may have more than $L6 sponsored Laws in the Edicts or in the queue or they will suffer sanctions on Tax</t>
-  </si>
-  <si>
-    <t>Each Player must have a Leader with at least level $L6 or they will suffer sanctions on Sue</t>
-  </si>
-  <si>
-    <t>No Player may have a Leader higher than level $L6 or they will suffer sanctions on Sue</t>
-  </si>
-  <si>
-    <t>Each Player must Collect at least $L6 Commodities this round or they will suffer sanctions on Recruit</t>
-  </si>
-  <si>
-    <t>No Player may Collect more than $L6 Commodities this round or they will suffer sanctions on Recruit</t>
-  </si>
-  <si>
-    <t>Each Player must have at least 3 + $L6 Leaders or they will suffer sanctions on Build &amp; Upgrade</t>
-  </si>
-  <si>
-    <t>No Player may have more than 3 + $L6 Leaders or they will suffer sanctions on Build &amp; Upgrade</t>
-  </si>
-  <si>
-    <t>Each Player must have at least $L6 Troops or they will suffer sanctions on Collect</t>
-  </si>
-  <si>
-    <t>No Player may have more than $L6 Troops or they will suffer sanctions on Collect</t>
-  </si>
-  <si>
-    <t>At least $L6 Players must use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
-  </si>
-  <si>
-    <t>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions on Prioritize</t>
-  </si>
-  <si>
-    <t>At least $L6 Players must use Court Actions or all Players suffer sanctions on Flatter</t>
-  </si>
-  <si>
-    <t>No more than $L6 Players may use Court Actions or all Players suffer sanctions on Flatter</t>
-  </si>
-  <si>
-    <t>Each Player must have at least $L6 Cards of each type in hand or they will suffer sanctions on Monetize</t>
-  </si>
-  <si>
-    <t>No Player may have more than $L6 Cards of each type in their hand or they will suffer sanctions on Monetize</t>
-  </si>
-  <si>
-    <t>Each Player must Deploy at least $L6 Troops or they will suffer sanctions on Donate</t>
-  </si>
-  <si>
-    <t>No Player may Deploy more than $L6 Troops or they will suffer sanctions on Donate</t>
-  </si>
-  <si>
-    <t>Each Player must Donate at least $L6 Coins or they will suffer sanctions on Postpone &amp; Prioritize</t>
-  </si>
-  <si>
-    <t>No Player may Donate more than $L6 Coins or they will suffer sanctions on Postpone &amp; Prioritize</t>
-  </si>
-  <si>
-    <t>Each Player must Sue using a Leader with at least level $L6 this round or they will suffer sanctions on Deploy</t>
-  </si>
-  <si>
-    <t>No Player may Sue using a Leader higher than level $L6 this round or they will suffer sanctions on Deploy</t>
-  </si>
-  <si>
-    <t>Each Player must have an Investment with at least level $L6 or they will suffer sanctions on Infiltrate</t>
-  </si>
-  <si>
-    <t>No Player may have an Investment higher than level $L6 or they will suffer sanctions on Infiltrate</t>
+    <t>The Royal Bank must have at least $L6 Coins or all Players suffer sanctions</t>
+  </si>
+  <si>
+    <t>The Royal Bank may not have more than $L6 Coins or all Players suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have at least 3 + $L6 Investments or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have more than 3 + $L6 Investments or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must Sue using a Leader with at least level $L6 this round or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may Sue using a Leader higher than level $L6 this round or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have an Investment with at least level $L6 or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have an Investment higher than level $L6 or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must deploy at least $L6 Troops or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may deploy more than $L6 Troops or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have at least $L6 sponsored Laws in the Edicts or in the Queue or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have more than $L6 sponsored Laws in the Edicts or in the queue or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have a Leader with at least level $L6 or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have a Leader higher than level $L6 or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must Collect at least $L6 Commodities this round or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may Collect more than $L6 Commodities this round or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have at least 3 + $L6 Leaders or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have more than 3 + $L6 Leaders or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have at least $L6 Troops or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have more than $L6 Troops or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>At least $L6 Players must use Undermarket Actions or all Players suffer sanctions</t>
+  </si>
+  <si>
+    <t>No more than $L6 Players may use Undermarket Actions or all Players suffer sanctions</t>
+  </si>
+  <si>
+    <t>At least $L6 Players must use Court Actions or all Players suffer sanctions</t>
+  </si>
+  <si>
+    <t>No more than $L6 Players may use Court Actions or all Players suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must have at least $L6 Cards of each type in hand or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may have more than $L6 Cards of each type in their hand or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must Deploy at least $L6 Troops or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may Deploy more than $L6 Troops or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>Each Player must Donate at least $L6 Coins or they will suffer sanctions</t>
+  </si>
+  <si>
+    <t>No Player may Donate more than $L6 Coins or they will suffer sanctions</t>
   </si>
 </sst>
 </file>
@@ -877,6 +877,10 @@
     </a>
   </bag>
 </FeaturePropertyBags>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1261,7 +1265,7 @@
       <c r="H2" s="2"/>
       <c r="I2" s="10"/>
     </row>
-    <row r="3" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>117</v>
       </c>
@@ -1433,7 +1437,7 @@
         <v>148</v>
       </c>
       <c r="D10" s="9" t="s">
-        <v>236</v>
+        <v>214</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>141</v>
@@ -1456,7 +1460,7 @@
         <v>23</v>
       </c>
       <c r="D11" s="9" t="s">
-        <v>237</v>
+        <v>215</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>145</v>
@@ -1479,7 +1483,7 @@
         <v>26</v>
       </c>
       <c r="D12" s="9" t="s">
-        <v>238</v>
+        <v>216</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>24</v>
@@ -1502,7 +1506,7 @@
         <v>28</v>
       </c>
       <c r="D13" s="9" t="s">
-        <v>239</v>
+        <v>217</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>27</v>
@@ -1514,7 +1518,7 @@
       <c r="H13" s="2"/>
       <c r="I13" s="10"/>
     </row>
-    <row r="14" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A14" s="8" t="s">
         <v>34</v>
       </c>
@@ -1525,7 +1529,7 @@
         <v>30</v>
       </c>
       <c r="D14" s="9" t="s">
-        <v>214</v>
+        <v>218</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>22</v>
@@ -1537,7 +1541,7 @@
       <c r="H14" s="3"/>
       <c r="I14" s="10"/>
     </row>
-    <row r="15" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A15" s="8" t="s">
         <v>152</v>
       </c>
@@ -1548,7 +1552,7 @@
         <v>32</v>
       </c>
       <c r="D15" s="9" t="s">
-        <v>215</v>
+        <v>219</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>33</v>
@@ -1560,7 +1564,7 @@
       <c r="H15" s="3"/>
       <c r="I15" s="10"/>
     </row>
-    <row r="16" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A16" s="8" t="s">
         <v>36</v>
       </c>
@@ -1571,7 +1575,7 @@
         <v>35</v>
       </c>
       <c r="D16" s="9" t="s">
-        <v>216</v>
+        <v>220</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>134</v>
@@ -1583,7 +1587,7 @@
       <c r="H16" s="2"/>
       <c r="I16" s="10"/>
     </row>
-    <row r="17" spans="1:9" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:9" ht="45" x14ac:dyDescent="0.25">
       <c r="A17" s="8" t="s">
         <v>39</v>
       </c>
@@ -1594,7 +1598,7 @@
         <v>37</v>
       </c>
       <c r="D17" s="9" t="s">
-        <v>217</v>
+        <v>221</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>131</v>
@@ -1617,7 +1621,7 @@
         <v>38</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>218</v>
+        <v>222</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>19</v>
@@ -1640,7 +1644,7 @@
         <v>40</v>
       </c>
       <c r="D19" s="9" t="s">
-        <v>219</v>
+        <v>223</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>127</v>
@@ -1663,7 +1667,7 @@
         <v>42</v>
       </c>
       <c r="D20" s="9" t="s">
-        <v>220</v>
+        <v>224</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>128</v>
@@ -1686,7 +1690,7 @@
         <v>44</v>
       </c>
       <c r="D21" s="9" t="s">
-        <v>221</v>
+        <v>225</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>132</v>
@@ -1709,7 +1713,7 @@
         <v>46</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>222</v>
+        <v>226</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>16</v>
@@ -1721,7 +1725,7 @@
       <c r="H22" s="3"/>
       <c r="I22" s="10"/>
     </row>
-    <row r="23" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A23" s="8" t="s">
         <v>150</v>
       </c>
@@ -1732,12 +1736,12 @@
         <v>48</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>223</v>
+        <v>227</v>
       </c>
       <c r="E23" s="10"/>
       <c r="F23" s="3"/>
     </row>
-    <row r="24" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A24" s="8" t="s">
         <v>151</v>
       </c>
@@ -1748,12 +1752,12 @@
         <v>50</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>224</v>
+        <v>228</v>
       </c>
       <c r="E24" s="10"/>
       <c r="F24" s="3"/>
     </row>
-    <row r="25" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A25" s="8" t="s">
         <v>53</v>
       </c>
@@ -1764,7 +1768,7 @@
         <v>51</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>225</v>
+        <v>229</v>
       </c>
       <c r="E25" s="10"/>
       <c r="F25" s="3"/>
@@ -1780,7 +1784,7 @@
         <v>52</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>226</v>
+        <v>230</v>
       </c>
       <c r="E26" s="10"/>
       <c r="F26" s="3"/>
@@ -1796,12 +1800,12 @@
         <v>54</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>227</v>
+        <v>231</v>
       </c>
       <c r="E27" s="10"/>
       <c r="F27" s="3"/>
     </row>
-    <row r="28" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A28" s="8" t="s">
         <v>59</v>
       </c>
@@ -1812,7 +1816,7 @@
         <v>56</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>228</v>
+        <v>232</v>
       </c>
       <c r="E28" s="10"/>
       <c r="F28" s="3"/>
@@ -1828,7 +1832,7 @@
         <v>58</v>
       </c>
       <c r="D29" s="9" t="s">
-        <v>229</v>
+        <v>233</v>
       </c>
       <c r="E29" s="10"/>
       <c r="F29" s="3"/>
@@ -1844,7 +1848,7 @@
         <v>60</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>230</v>
+        <v>234</v>
       </c>
       <c r="E30" s="10"/>
       <c r="F30" s="3"/>
@@ -1860,12 +1864,12 @@
         <v>62</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>231</v>
+        <v>235</v>
       </c>
       <c r="E31" s="10"/>
       <c r="F31" s="3"/>
     </row>
-    <row r="32" spans="1:9" ht="45" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:9" ht="30" x14ac:dyDescent="0.25">
       <c r="A32" s="8" t="s">
         <v>65</v>
       </c>
@@ -1876,12 +1880,12 @@
         <v>125</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>232</v>
+        <v>236</v>
       </c>
       <c r="E32" s="10"/>
       <c r="F32" s="3"/>
     </row>
-    <row r="33" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="33" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A33" s="8" t="s">
         <v>66</v>
       </c>
@@ -1892,12 +1896,12 @@
         <v>126</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>233</v>
+        <v>237</v>
       </c>
       <c r="E33" s="10"/>
       <c r="F33" s="3"/>
     </row>
-    <row r="34" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A34" s="8" t="s">
         <v>116</v>
       </c>
@@ -1908,12 +1912,12 @@
         <v>153</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>234</v>
+        <v>238</v>
       </c>
       <c r="E34" s="10"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="1:6" ht="45" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:6" ht="30" x14ac:dyDescent="0.25">
       <c r="A35" s="8" t="s">
         <v>123</v>
       </c>
@@ -1924,7 +1928,7 @@
         <v>154</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>235</v>
+        <v>239</v>
       </c>
       <c r="E35" s="10"/>
       <c r="F35" s="3"/>

</xml_diff>